<commit_message>
Scale affiliate recruitment 10x — Power Affiliate recruits 5,000 by Year 5
- Year 1-3: 50/250/1,000 (was 5/25/100)
- Year 4: 100/500/2,500 (was 10/50/250)
- Year 5: 200/1,000/5,000 (was 20/100/500)
- Updated both web page and downloadable xlsx
</commit_message>
<xml_diff>
--- a/public/SearchStar_Revenue_Projections.xlsx
+++ b/public/SearchStar_Revenue_Projections.xlsx
@@ -2400,13 +2400,13 @@
         <v>94</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>25</v>
+        <v>250</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2448,15 +2448,15 @@
       </c>
       <c r="B12" s="23" t="n">
         <f aca="false">B7*B8*B9</f>
-        <v>2.5</v>
+        <v>25</v>
       </c>
       <c r="C12" s="23" t="n">
         <f aca="false">C7*C8*C9</f>
-        <v>25</v>
+        <v>250</v>
       </c>
       <c r="D12" s="23" t="n">
         <f aca="false">D7*D8*D9</f>
-        <v>150</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2470,15 +2470,15 @@
       </c>
       <c r="B15" s="28" t="n">
         <f aca="false">B12*12</f>
-        <v>30</v>
+        <v>300</v>
       </c>
       <c r="C15" s="28" t="n">
         <f aca="false">C12*12</f>
-        <v>300</v>
+        <v>3000</v>
       </c>
       <c r="D15" s="28" t="n">
         <f aca="false">D12*12</f>
-        <v>1800</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2491,13 +2491,13 @@
         <v>102</v>
       </c>
       <c r="B18" s="7" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>250</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2520,15 +2520,15 @@
       </c>
       <c r="B20" s="29" t="n">
         <f aca="false">B18*B19*0.05*12</f>
-        <v>180</v>
+        <v>1800</v>
       </c>
       <c r="C20" s="29" t="n">
         <f aca="false">C18*C19*0.05*12</f>
-        <v>1500</v>
+        <v>15000</v>
       </c>
       <c r="D20" s="29" t="n">
         <f aca="false">D18*D19*0.05*12</f>
-        <v>12000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2536,13 +2536,13 @@
         <v>105</v>
       </c>
       <c r="B22" s="7" t="n">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2565,15 +2565,15 @@
       </c>
       <c r="B24" s="28" t="n">
         <f aca="false">B22*B23*0.05*12</f>
-        <v>600</v>
+        <v>6000</v>
       </c>
       <c r="C24" s="28" t="n">
         <f aca="false">C22*C23*0.05*12</f>
-        <v>4800</v>
+        <v>48000</v>
       </c>
       <c r="D24" s="28" t="n">
         <f aca="false">D22*D23*0.05*12</f>
-        <v>36000</v>
+        <v>360000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>